<commit_message>
fixes l interfaces, w zdt bl l tables ta3 agent, w bdelt alerts b toast
</commit_message>
<xml_diff>
--- a/my-app/server/test.xlsx
+++ b/my-app/server/test.xlsx
@@ -428,22 +428,22 @@
     </row>
     <row r="2">
       <c r="A2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B2" t="str">
-        <v>Sara Ahmed</v>
+        <v>Ali Bensaid</v>
       </c>
       <c r="C2" t="str">
-        <v>C124</v>
+        <v>C125</v>
       </c>
       <c r="D2" t="str">
-        <v>BL002</v>
+        <v>BL003</v>
       </c>
       <c r="E2" t="str">
-        <v>TX1002</v>
+        <v>TX1003</v>
       </c>
       <c r="F2" t="str">
-        <v>250.00</v>
+        <v>75.00</v>
       </c>
       <c r="G2" s="1">
         <v>46109.000243055554</v>
@@ -454,25 +454,25 @@
     </row>
     <row r="3">
       <c r="A3">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="B3" t="str">
-        <v>Ali Bensaid</v>
+        <v>Yanis Amrani</v>
       </c>
       <c r="C3" t="str">
-        <v>C125</v>
+        <v>C123</v>
       </c>
       <c r="D3" t="str">
-        <v>BL003</v>
+        <v>BL001</v>
       </c>
       <c r="E3" t="str">
-        <v>TX1003</v>
+        <v>TX1001</v>
       </c>
       <c r="F3" t="str">
-        <v>75.00</v>
+        <v>120.00</v>
       </c>
       <c r="G3" s="1">
-        <v>46109.000243055554</v>
+        <v>46108.000243055554</v>
       </c>
       <c r="H3" t="str">
         <v>approved</v>
@@ -480,28 +480,28 @@
     </row>
     <row r="4">
       <c r="A4">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="B4" t="str">
-        <v>Yanis Amrani</v>
+        <v>Sara Ahmed</v>
       </c>
       <c r="C4" t="str">
-        <v>C123</v>
+        <v>C124</v>
       </c>
       <c r="D4" t="str">
-        <v>BL001</v>
+        <v>BL002</v>
       </c>
       <c r="E4" t="str">
-        <v>TX1001</v>
+        <v>TX1002</v>
       </c>
       <c r="F4" t="str">
-        <v>120.00</v>
+        <v>250.00</v>
       </c>
       <c r="G4" s="1">
-        <v>46108.000243055554</v>
+        <v>46109.000243055554</v>
       </c>
       <c r="H4" t="str">
-        <v>Pending</v>
+        <v>approved</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix l status w buttons reject w approved ki ykono disabled
</commit_message>
<xml_diff>
--- a/my-app/server/test.xlsx
+++ b/my-app/server/test.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -428,12 +428,12 @@
     </row>
     <row r="2">
       <c r="A2">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="B2" t="str">
         <v>Mourad</v>
       </c>
-      <c r="C2">
+      <c r="C2" t="str">
         <v>10</v>
       </c>
       <c r="D2" t="str">
@@ -449,12 +449,64 @@
         <v>46120.000243055554</v>
       </c>
       <c r="H2" t="str">
-        <v>approved</v>
+        <v>pending</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3">
+        <v>21</v>
+      </c>
+      <c r="B3" t="str">
+        <v>imad</v>
+      </c>
+      <c r="C3" t="str">
+        <v>1</v>
+      </c>
+      <c r="D3" t="str">
+        <v>BL-10045</v>
+      </c>
+      <c r="E3" t="str">
+        <v>tr345</v>
+      </c>
+      <c r="F3" t="str">
+        <v>2000.00</v>
+      </c>
+      <c r="G3" s="1">
+        <v>36899.000243055554</v>
+      </c>
+      <c r="H3" t="str">
+        <v>pending</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4">
+        <v>22</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Yanis Amrani</v>
+      </c>
+      <c r="C4" t="str">
+        <v>C123</v>
+      </c>
+      <c r="D4" t="str">
+        <v>BL001</v>
+      </c>
+      <c r="E4" t="str">
+        <v>TX1001</v>
+      </c>
+      <c r="F4" t="str">
+        <v>120.00</v>
+      </c>
+      <c r="G4" s="1">
+        <v>46108.000243055554</v>
+      </c>
+      <c r="H4" t="str">
+        <v>pending</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
function li t9ra excel file f placat csv
</commit_message>
<xml_diff>
--- a/my-app/server/test.xlsx
+++ b/my-app/server/test.xlsx
@@ -428,7 +428,7 @@
     </row>
     <row r="2">
       <c r="A2">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="B2" t="str">
         <v>Mourad</v>
@@ -454,13 +454,13 @@
     </row>
     <row r="3">
       <c r="A3">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="B3" t="str">
         <v>imad</v>
       </c>
       <c r="C3" t="str">
-        <v>1</v>
+        <v>01</v>
       </c>
       <c r="D3" t="str">
         <v>BL-10045</v>
@@ -480,7 +480,7 @@
     </row>
     <row r="4">
       <c r="A4">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="B4" t="str">
         <v>Yanis Amrani</v>

</xml_diff>